<commit_message>
Updated the New working models and deleted depricated models
</commit_message>
<xml_diff>
--- a/LLM Final Output.xlsx
+++ b/LLM Final Output.xlsx
@@ -1461,7 +1461,8 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>b. City name available but main city not matching</t>
+          <t xml:space="preserve">Error: 503 - {"error":{"message":"qwen/qwen3.8-27b is currently over capacity. Please try again and back off exponentially. Visit https://groqstatus.com to see if there is an active incident.","type":"internal_server_error"}}
+</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1916,7 +1917,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>b. City name available but main city not matching</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1926,7 +1927,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2266,8 +2267,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 1.008999999s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2317,8 +2317,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 1.992s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2328,7 +2327,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2418,8 +2417,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 1.664s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>b. City name available but main city not matching</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2469,8 +2467,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 1.591s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2520,8 +2517,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 147ms. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2531,7 +2527,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2571,8 +2567,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 1.95s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2582,7 +2577,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2622,8 +2617,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 1.996s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2633,7 +2627,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2723,8 +2717,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 1.976s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2734,7 +2727,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2774,8 +2767,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: 429 - {"error":{"message":"Rate limit reached for model `llama-3.3-70b-versatile` in organization `org_01k56kcx4jf4dsjbw4w0d4sbrn` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 868ms. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing","type":"requests","code":"rate_limit_exceeded"}}
-</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2785,7 +2777,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2817,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>b. City name available but main city not matching</t>
+          <t>a. City name available and main city matching</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2835,7 +2827,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Result_Model2 is wrong</t>
+          <t>Correct</t>
         </is>
       </c>
     </row>

</xml_diff>